<commit_message>
commando: Physiocure audit + reply messages; first yes logged in the lead sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PegPysKFWvspoEqHMUg1m9
</commit_message>
<xml_diff>
--- a/commando/leads/leads-2026-10-11.xlsx
+++ b/commando/leads/leads-2026-10-11.xlsx
@@ -790,11 +790,19 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>Not called</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
+          <t>Replied yes (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>18 Oct: said yes to the audit on WhatsApp. Audit PDF sent.</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Physiocure+Egypt+Zahraa+El+Maadi</t>
@@ -10375,9 +10383,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -10392,9 +10398,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -10430,9 +10434,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
@@ -10482,9 +10484,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
@@ -10534,9 +10534,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
@@ -10600,9 +10598,7 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
@@ -10666,9 +10662,7 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-    </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
@@ -10711,9 +10705,7 @@
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
@@ -10749,9 +10741,7 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-    </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -10822,9 +10812,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-    </row>
+    <row r="71"/>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
@@ -10895,9 +10883,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-    </row>
+    <row r="82"/>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
@@ -10912,9 +10898,7 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-    </row>
+    <row r="85"/>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
@@ -10950,9 +10934,7 @@
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr"/>
-    </row>
+    <row r="91"/>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>

</xml_diff>